<commit_message>
feat: add frontend dashboard, implement robust error handling, and update RPA data records
</commit_message>
<xml_diff>
--- a/reporte_supermercados.xlsx
+++ b/reporte_supermercados.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="129">
   <si>
     <t>🛒 REPORTE RPA: COMPARADOR DE PRECIOS Y CANASTA INTELIGENTE</t>
   </si>
@@ -351,14 +351,14 @@
     <t>🎯 CONSULTA INDIVIDUAL: ¿DÓNDE TE CONVIENE COMPRAR?</t>
   </si>
   <si>
-    <t>🔎 PRODUCTO CONSULTADO:  "LECHE"</t>
-  </si>
-  <si>
-    <t>Intención detectada: GENERICA  │  Fecha: 2026-09-10  │  Supermercados relevados: Carrefour, COTO y Día %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">🏆 TE CONVIENE COMPRAR EN: COTO ($ 2.140,00)
-💰 AHORRO POTENCIAL: $ 200,00 (9% menos que en Carrefour)</t>
+    <t>🔎 PRODUCTO CONSULTADO:  "MAYONESA NATURA"</t>
+  </si>
+  <si>
+    <t>Intención detectada: ESPECIFICA (Marca: NATURA)  │  Fecha: 2026-09-10  │  Supermercados relevados: Carrefour, COTO y Día %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">🏆 TE CONVIENE COMPRAR EN: Carrefour ($ 3.039,00)
+💰 AHORRO POTENCIAL: $ 3,00 (0% menos que en COTO)</t>
   </si>
   <si>
     <t>Precio Vigente</t>
@@ -376,31 +376,28 @@
     <t>Enlace Web Directo</t>
   </si>
   <si>
+    <t>🏆 GANADOR</t>
+  </si>
+  <si>
+    <t>Mayonesa Natura 475 g.</t>
+  </si>
+  <si>
+    <t>Coincidencia específica validada (marca, categoría y atributos conformes).</t>
+  </si>
+  <si>
+    <t>🔗 Ver en Carrefour</t>
+  </si>
+  <si>
     <t xml:space="preserve"> VALIDADA</t>
   </si>
   <si>
-    <t>Leche Protein La Serenisima 1L</t>
-  </si>
-  <si>
-    <t>Coincidencia genérica validada (alternativa comercial aceptable).</t>
-  </si>
-  <si>
-    <t>🔗 Ver en Carrefour</t>
-  </si>
-  <si>
-    <t>🏆 GANADOR</t>
-  </si>
-  <si>
-    <t>Leche Multidefensas 3% LA SERENISIMA Sachet 1l</t>
+    <t>Mayonesa NATURA Pouch 475 Gr</t>
   </si>
   <si>
     <t>🔗 Ver en COTO</t>
   </si>
   <si>
-    <t>N/D</t>
-  </si>
-  <si>
-    <t>❌ NO ENCONTRADO</t>
+    <t>Mayonesa Natura 500 Ml.</t>
   </si>
   <si>
     <t>🔗 Ver en Día %</t>
@@ -416,7 +413,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="40" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -558,6 +555,29 @@
     </font>
     <font>
       <b/>
+      <color rgb="276A3C"/>
+      <sz val="10"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="276A3C"/>
+      <sz val="9.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <color rgb="FF444444"/>
+      <sz val="8.5"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0563C1"/>
+      <sz val="9"/>
+      <name val="Segoe UI"/>
+    </font>
+    <font>
+      <b/>
       <color rgb="FF333333"/>
       <sz val="9.5"/>
       <name val="Segoe UI"/>
@@ -573,54 +593,13 @@
       <name val="Segoe UI"/>
     </font>
     <font>
-      <color rgb="FF444444"/>
-      <sz val="8.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0563C1"/>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="276A3C"/>
-      <sz val="10"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="276A3C"/>
-      <sz val="9.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF888888"/>
-      <strike/>
-      <sz val="9.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="C00000"/>
-      <sz val="9"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
-      <color rgb="C00000"/>
-      <sz val="8.5"/>
-      <name val="Segoe UI"/>
-    </font>
-    <font>
       <i/>
       <color rgb="FF666666"/>
       <sz val="9"/>
       <name val="Segoe UI"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -667,11 +646,6 @@
         <fgColor rgb="FCE4D6"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF9EAE1"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -700,7 +674,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -821,52 +795,43 @@
     <xf numFmtId="0" fontId="27" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="34" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="34" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1208,7 +1173,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H35"/>
+  <dimension ref="B2:H34"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -1735,29 +1700,6 @@
         <v>91</v>
       </c>
       <c r="H34" s="23" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B35" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="C35" s="27" t="s">
-        <v>22</v>
-      </c>
-      <c r="D35" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="E35" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="G35" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="H35" s="23" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1788,7 +1730,6 @@
     <hyperlink ref="H24" r:id="rId9"/>
     <hyperlink ref="H33" r:id="rId10"/>
     <hyperlink ref="H34" r:id="rId11"/>
-    <hyperlink ref="H35" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -2177,7 +2118,7 @@
         <v>6</v>
       </c>
       <c r="C11" s="43">
-        <v>2340</v>
+        <v>3039</v>
       </c>
       <c r="D11" s="44" t="s">
         <v>119</v>
@@ -2197,7 +2138,7 @@
         <v>19</v>
       </c>
       <c r="C12" s="49">
-        <v>2140</v>
+        <v>3042</v>
       </c>
       <c r="D12" s="50" t="s">
         <v>123</v>
@@ -2213,34 +2154,34 @@
       </c>
     </row>
     <row r="13" ht="26" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" s="42" t="s">
+      <c r="B13" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="C13" s="54" t="s">
+      <c r="C13" s="49">
+        <v>3040</v>
+      </c>
+      <c r="D13" s="50" t="s">
+        <v>123</v>
+      </c>
+      <c r="E13" s="51" t="s">
         <v>126</v>
       </c>
-      <c r="D13" s="55" t="s">
+      <c r="F13" s="52" t="s">
+        <v>121</v>
+      </c>
+      <c r="G13" s="53" t="s">
         <v>127</v>
       </c>
-      <c r="E13" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" s="56" t="s">
-        <v>86</v>
-      </c>
-      <c r="G13" s="47" t="s">
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="54" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="57" t="s">
-        <v>129</v>
-      </c>
-      <c r="C15" s="57"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="57"/>
-      <c r="G15" s="57"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="54"/>
+      <c r="E15" s="54"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>